<commit_message>
Update index: 1280 → 1685 | 20 businesses found (scan 21-07-2026)
Scanned addresses from index 1280 (איסלנד 12) to 1684 (אסתר המלכה 2).
Found 20 verified businesses across multiple Jerusalem streets.
Added Excel report: דוח נכסים לתאריך:21-07-2026.xlsx
</commit_message>
<xml_diff>
--- a/דוח נכסים לתאריך:21-07-2026.xlsx
+++ b/דוח נכסים לתאריך:21-07-2026.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,12 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -46,23 +52,20 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
-        <bgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -70,20 +73,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="thin">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -450,19 +473,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -499,20 +522,20 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>רקמת רוזנפלד</t>
+          <t>מכללת ש"ש-האקדמיה לשיווק שותפים</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>אדניהו הכהן 40, ירושלים</t>
+          <t>איסלנד 17, ירושלים</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>רקמה וטקסטיל</t>
+          <t>קורסים והשתלמויות</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -520,57 +543,57 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80159027/18920/</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80181095/8190/</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>סרטי סקופוס ירושלים (1987) בע"מ</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>אהל משה 7, ירושלים</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>הפקות קולנוע וטלוויזיה</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/38057100/36840/</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>רונית שקלים</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>איסלנד 17, ירושלים</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>גרפיקאים וסטודיו לגרפיקה</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80027963/11301/</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>מינימרקט טופן יוסף</t>
+          <t>מוטי רבינוביץ מאמן כושר אישי</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>אודם 580, ירושלים</t>
+          <t>איסלנד 21, ירושלים</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>סופרמרקט / מכולת</t>
+          <t>מדריכי ספורט וכושר</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -578,57 +601,57 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/37799980/35760/</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80272956/22570/</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>נוראל הנדסה ואדריכלות</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>אודם 580, ירושלים</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>מהנדסי בנייה וקונסטרוקציות</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80052505/23755/</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>יעל פרץ-מורה לצרפתית</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>אלעזר המודעי 12, ירושלים</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>שיעורים פרטיים</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80015963/24630/</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>יעקבי ששון</t>
+          <t>גלעד גלי - שרה עו"ד</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>אוליפנט 2, ירושלים</t>
+          <t>אלפסי 21, ירושלים</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>עיתונאים</t>
+          <t>עורכי דין פלילי</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -636,57 +659,57 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/6026560/38190/</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/27624410/9010106/</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>המרכז לריהוט משרדי</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>אולשן יצחק 15, ירושלים</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>ריהוט משרדי</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80070952/45750/</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>עו"ד חוה ולר</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>אלפנדרי 36, ירושלים</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>עורכי דין - דיני מקרקעין</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80231621/9010118/</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ד"ר ליפשיץ יצחק</t>
+          <t>מזיקיס-המדביר היווני</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>אורוגואי 12, ירושלים</t>
+          <t>אלפנדרי 6, ירושלים</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>רופא כללי</t>
+          <t>הדברה</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -694,15 +717,414 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/6827160/46350/</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80182149/13110/</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>המכון לעסקאות עתידיות ואופציות בע"מ</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>אלפסי 23, ירושלים</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>יועצי השקעות</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/25760070/14400/</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>שטרנגר גבי</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>אלקחי מרדכי 20, ירושלים</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>פסיכולוגים קליניים</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/60148150/40270/</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>דריבן שירותי אבטחה ואימונים</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>אלקחי מרדכי 38, ירושלים</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>שמירה ואבטחה</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80014328/49230/</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>שרית מהגר אמנות האיפור</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>אלקחי מרדכי 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>איפור</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80054059/2800/</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>עו"ד גבאי דניאל</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>אמיל זולא 6, ירושלים</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>עורכי דין - דיני מקרקעין</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80276756/9010118/</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ארנסקי אבי</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>אמיל זולא 6, ירושלים</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>תרגום</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/75711850/51870/</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>יתד התחדשות עירונית</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>אמיל זולא 6, ירושלים</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>נדל"ן - התחדשות עירונית</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80243217/34590/</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ענת לביא</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>אמציה 8, ירושלים</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>פסיכותרפיה</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80102167/40230/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>לוי יוסי הובלות והרכבות</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>אנטיגנוס 11, ירושלים</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>חברות הובלה ומובילים</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80032602/35840/</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>גולן עליזה</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>אנילביץ 64, ירושלים</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>פלדנקרייז - טיפול בתנועה</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80065084/40030014/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>גן האור - גן אנתרופוסופי</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>אנילביץ 26, ירושלים</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>גני ילדים</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80108035/10880/</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>כהן אמנון</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>אנילביץ 68, ירושלים</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>מורה לנהיגה</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/24466980/8450/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>נלפ ישראל</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>אסתר המלכה 2, ירושלים</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>אבחון וטיפול בלקויי למידה</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80166202/22310/</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>